<commit_message>
fix: repair notebook 2 syntax and update results with Jaime Ramos Miranda as sole author
</commit_message>
<xml_diff>
--- a/artifacts/cuadros_fenotipos.xlsx
+++ b/artifacts/cuadros_fenotipos.xlsx
@@ -10,12 +10,12 @@
     <sheet name="Variables continuas" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Variables binarias pct" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Mortalidad" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Centroides" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Sexo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Anemia" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Diabetes" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Hipertension" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Tabaquismo" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="anaemia" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="diabetes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="high_blood_pressure" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="sex" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="smoking" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="DEATH_EVENT" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -728,7 +728,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>tasa_mortalidad_%</t>
+          <t>tasa_%</t>
         </is>
       </c>
     </row>
@@ -799,241 +799,128 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>fenotipo</t>
+        </is>
+      </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>age</t>
+          <t>anaemia</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>anaemia</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>creatinine_phosphokinase</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>diabetes</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>ejection_fraction</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>high_blood_pressure</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>platelets</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>serum_creatinine</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>serum_sodium</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>sex</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>smoking</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>time</t>
+          <t>Freq</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Fenotipo 1</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>-0.03157507873377631</v>
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>0.06527658522323368</v>
-      </c>
-      <c r="D2" t="n">
-        <v>-0.1475500548207281</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.063285927004609</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.09228082229489697</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1.35927151357595</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.05656448611897233</v>
-      </c>
-      <c r="I2" t="n">
-        <v>-0.2779569467399815</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.08174384443122679</v>
-      </c>
-      <c r="K2" t="n">
-        <v>-0.539504672914165</v>
-      </c>
-      <c r="L2" t="n">
-        <v>-0.6255995117752017</v>
-      </c>
-      <c r="M2" t="n">
-        <v>-0.1700203965284134</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Fenotipo 2</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>-0.09793823616224027</v>
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>-0.1554842101978103</v>
-      </c>
-      <c r="D3" t="n">
-        <v>-0.1164505897454442</v>
-      </c>
-      <c r="E3" t="n">
-        <v>-0.2059939757835371</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-0.03171817344701507</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-0.125763213248773</v>
-      </c>
-      <c r="H3" t="n">
-        <v>-0.02914048002719754</v>
-      </c>
-      <c r="I3" t="n">
-        <v>-0.2189802009645894</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.1712401716591614</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.7356881903374962</v>
-      </c>
-      <c r="L3" t="n">
-        <v>1.454160697217931</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.1598349410151179</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Fenotipo 3</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>-0.3297181688200573</v>
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
       <c r="C4" t="n">
-        <v>0.04869483196537774</v>
-      </c>
-      <c r="D4" t="n">
-        <v>-0.05469792533136503</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.2787594403774443</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.2176839806357227</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-0.7356881903374968</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.01687703745846632</v>
-      </c>
-      <c r="I4" t="n">
-        <v>-0.2112872189671602</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.2666418405348024</v>
-      </c>
-      <c r="K4" t="n">
-        <v>-0.4747329719236044</v>
-      </c>
-      <c r="L4" t="n">
-        <v>-0.6876819060735041</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.4063219384727984</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Fenotipo 4</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>0.9141125066538007</v>
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
       </c>
       <c r="C5" t="n">
-        <v>0.07112896872600619</v>
-      </c>
-      <c r="D5" t="n">
-        <v>-0.1980224817216552</v>
-      </c>
-      <c r="E5" t="n">
-        <v>-0.3519902987684916</v>
-      </c>
-      <c r="F5" t="n">
-        <v>-0.5938997461028015</v>
-      </c>
-      <c r="G5" t="n">
-        <v>-0.3166962495548083</v>
-      </c>
-      <c r="H5" t="n">
-        <v>-0.3504835221027117</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.5817190925819672</v>
-      </c>
-      <c r="J5" t="n">
-        <v>-0.691844805933318</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.5029148899026702</v>
-      </c>
-      <c r="L5" t="n">
-        <v>-0.306909887710582</v>
-      </c>
-      <c r="M5" t="n">
-        <v>-0.6297301111461622</v>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1047,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1058,7 +945,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>sex</t>
+          <t>diabetes</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -1073,11 +960,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>hombre</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3">
@@ -1086,11 +973,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>mujer</t>
+          <t>sí</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -1099,24 +986,24 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>hombre</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>79</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>hombre</t>
+          <t>sí</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
@@ -1125,24 +1012,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>mujer</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>52</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>hombre</t>
+          <t>sí</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8">
@@ -1151,11 +1038,24 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>mujer</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1169,7 +1069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1180,7 +1080,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>anaemia</t>
+          <t>high_blood_pressure</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -1195,24 +1095,24 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>sí</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>37</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>32</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4">
@@ -1221,29 +1121,29 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>sí</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>51</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>28</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1251,12 +1151,12 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>49</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1264,33 +1164,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1304,7 +1178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1315,7 +1189,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>diabetes</t>
+          <t>sex</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -1330,11 +1204,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>hombre</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>38</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
@@ -1343,11 +1217,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>mujer</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>31</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4">
@@ -1356,24 +1230,24 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>hombre</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>54</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>hombre</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6">
@@ -1382,24 +1256,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>mujer</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>hombre</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8">
@@ -1408,24 +1282,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>mujer</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1450,7 +1311,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>high_blood_pressure</t>
+          <t>smoking</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -1465,24 +1326,24 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>56</v>
       </c>
     </row>
     <row r="4">
@@ -1495,7 +1356,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>23</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5">
@@ -1521,7 +1382,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7">
@@ -1534,7 +1395,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1548,7 +1409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1559,7 +1420,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>smoking</t>
+          <t>DEATH_EVENT</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -1574,11 +1435,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>fallecido</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>67</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3">
@@ -1587,11 +1448,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>vivo</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4">
@@ -1600,50 +1461,76 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>fallecido</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>79</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>vivo</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>fallecido</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>37</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
         <v>4</v>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>8</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>fallecido</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>